<commit_message>
Uploading documentation for phase3
</commit_message>
<xml_diff>
--- a/documents/ITC327W_Project_Progress_Tracker_2026.xlsx
+++ b/documents/ITC327W_Project_Progress_Tracker_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mamel\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BC209D6-895F-4265-B0EB-03804E879135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2139D145-78E9-4CED-978A-245B1C381DE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1815" yWindow="1815" windowWidth="14010" windowHeight="11295" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -32,9 +32,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -103,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="437">
   <si>
     <t>ITC327W Project Progress and Contribution Workbook</t>
   </si>
@@ -597,9 +594,15 @@
     <t>Resolved</t>
   </si>
   <si>
+    <t>N/A</t>
+  </si>
+  <si>
     <t>All</t>
   </si>
   <si>
+    <t>We did not encounter major interpersonal conflicts, but external stakeholder delays and internal schedule delays and internal schedule mismatches disrupted our timelines. We adapted by rescheduling interviews, conducting asynchronous follow-ups, and redistributing critical drafting responsibilities to ensure project milestones and documentation requirements were met on time.</t>
+  </si>
+  <si>
     <t>Supabase setup &amp; SRS documentation</t>
   </si>
   <si>
@@ -852,9 +855,6 @@
     <t>Nothing</t>
   </si>
   <si>
-    <t>Improve good group communication and address participation cooncerns</t>
-  </si>
-  <si>
     <t>Project progress tracker and Microsoft project Scheduling</t>
   </si>
   <si>
@@ -969,21 +969,18 @@
     <t>Did the Sequence Diagram for Flutter</t>
   </si>
   <si>
+    <t>Did all the Documentation And also The Updated SRS</t>
+  </si>
+  <si>
+    <t>Updated the Project Tracker and Fixed the MS project Also Designed the System Architecture</t>
+  </si>
+  <si>
     <t>Completed the Sequence Diagram For the ASP.NET</t>
   </si>
   <si>
     <t>Completed the Sequence Diagram For the Flutter</t>
   </si>
   <si>
-    <t>7 September to 25 September</t>
-  </si>
-  <si>
-    <t>Updated the Complete SRS and The System Architecture and Design</t>
-  </si>
-  <si>
-    <t>Lerato Mahlatsi, Paballo Lebusa,Mamello Lepitla</t>
-  </si>
-  <si>
     <t>Did the Interface designs but they were incomplete and was finished by Mamello Lepitla and Paballo Lebusa</t>
   </si>
   <si>
@@ -993,21 +990,18 @@
     <t>Completed the Use Case for Both Parent and Admin and github Documentation</t>
   </si>
   <si>
+    <t>The Interface Design was left unfinished.</t>
+  </si>
+  <si>
+    <t>Some  Students had to leave they work and fix the design</t>
+  </si>
+  <si>
+    <t>A new interface design was done by some members</t>
+  </si>
+  <si>
     <t>Mamello lepitla, Paballo Lebusa</t>
   </si>
   <si>
-    <t>7- 25 September 2026</t>
-  </si>
-  <si>
-    <t>The System Architecture, ERD Table, Use Case Diagram, GitHub Documentation, Sequence Diagrams and Updated SRS Documentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Progress Tracker and Updated SRS </t>
-  </si>
-  <si>
-    <t>Developing the Prototypes</t>
-  </si>
-  <si>
     <t>Phehello Online Enrollments System</t>
   </si>
   <si>
@@ -1032,58 +1026,391 @@
     <t>Added a dedicated Payment Information screen displaying the fee and banking details and updated proof of payment screen to capture the payment reference before the proof of payment document is uploaded</t>
   </si>
   <si>
-    <t>Early design decisions shape everything that follows. Mapping the use cases, sequence diagrams and ERD before coding showed how the Flutter app, ASP.NET app and Supabase must fit together. It also exposed gaps in our Phase 1 schema, such as learner medical details and payment resubmissions, which we fixed on paper instead of in code.</t>
-  </si>
-  <si>
-    <t>The Flutter and ASP.NET interface designs were the hardest part. The first version was left incomplete, so the screens were rebuilt from scratch close to the deadline and the stakeholder's colour scheme was applied afterwards. This made our final submission late and put the assessment mark at risk. The sequence and use case diagrams were also complex, mainly the include/extend relationships.</t>
-  </si>
-  <si>
-    <t>The architecture, use case diagrams, sequence diagrams and ERD were completed as assigned. The stakeholder feedback loop also worked well. The secretary quickly confirmed the interface colours (brown and white) and the R200 fee and banking details, which became FR15 and a new Payment Information screen.</t>
-  </si>
-  <si>
-    <t>Tasks were assigned in Microsoft Project by strength: architecture, use case, sequence diagrams, ERD, interface designs, stakeholder feedback, documentation, and tracker and repository upkeep. Most tasks were completed as assigned, but the interface design task was not and had to be redone by other members.</t>
-  </si>
-  <si>
-    <t>Not fully. Most members completed their Phase 2 tasks. The interface designs assigned to Lerato Mahlatsi were incomplete. Mamello Lepitla rebuilt the screens from scratch with help from Paballo Lebusa, while also completing the SRS documentation. This is recorded in the Individual Contributions sheet.</t>
-  </si>
-  <si>
-    <t>There was no open conflict, but the incomplete designs caused our biggest delay. We reassigned the work to two members and held extra check-ins to finish. We should have raised the problem earlier instead of waiting until the deadline was close.</t>
-  </si>
-  <si>
-    <t>The stakeholder confirmed the payment step and the two staff roles. Small details, such as showing the fee and banking details before proof of payment, matter to real users. We also learned to confirm design choices like colours before building screens, not after.</t>
-  </si>
-  <si>
-    <t>Set internal check-in dates before every deadline. Each member must show progress halfway through their task and say at least two days before the due date if they are stuck, so unfinished work is reassigned early.</t>
-  </si>
-  <si>
-    <t>Split large deliverables into smaller tasks, keep work visible in the shared GitHub repository and Figma file, and confirm stakeholder requirements before building.</t>
-  </si>
-  <si>
-    <t>Test the Flutter, ASP.NET and Supabase connection first, then build the parent and staff features in small tasks, testing each integration point as it is built.</t>
-  </si>
-  <si>
-    <t>Yes – Flutter/ASP.NET interface designs were left incomplete and completed by two other members.</t>
-  </si>
-  <si>
-    <t>Completing the Flutter and ASP.NET interface designs on time after the first version was left incomplete.</t>
-  </si>
-  <si>
-    <t>Phase 3 – development, integration and testing</t>
-  </si>
-  <si>
-    <t>Flutter and ASP.NET interface designs were left incomplete.</t>
-  </si>
-  <si>
-    <t>Screens were rebuilt from scratch close to the deadline, causing a late submission.</t>
-  </si>
-  <si>
-    <t>Work reassigned to two members, stakeholder colour scheme applied, extra check-ins held</t>
-  </si>
-  <si>
-    <t>Updated SRS documentation and ERD; rebuilt the Flutter and ASP.NET screens from scratch and applied the stakeholder's brown and white colour scheme.</t>
-  </si>
-  <si>
-    <t>Updated the Project Tracker and Fixed the MS project Also Designed the System Architecture. Helped complete the Flutter and ASP.NET screens.</t>
+    <t>Unit 4 / Phase 3</t>
+  </si>
+  <si>
+    <t>28 September 2026 to 25 October 2026</t>
+  </si>
+  <si>
+    <t>Updated and completed the SRS and Developed and integrated the Flutter parent enrolment app and the ASP.NET staff web app on a shared Supabase backend, covering application submission, document and proof-of-payment upload, staff review, payment verification and confirmation letters.</t>
+  </si>
+  <si>
+    <t>Making both apps work safely on one Supabase database, because row-level security and file-storage rules blocked cross-role actions unti][</t>
+  </si>
+  <si>
+    <t>Phase 3 final  presentation</t>
+  </si>
+  <si>
+    <t>Confirmation letters</t>
+  </si>
+  <si>
+    <t>Delete application</t>
+  </si>
+  <si>
+    <t>Test data and sample documents</t>
+  </si>
+  <si>
+    <t>Integration and testing</t>
+  </si>
+  <si>
+    <t>Row-level security stopped staff and parents from doing what each role needed.</t>
+  </si>
+  <si>
+    <t>Some staff screens and uploads failed until access was fixed.</t>
+  </si>
+  <si>
+    <t>Wrote a staff access patch and per-role policies for tables and storage.</t>
+  </si>
+  <si>
+    <t>Paballo Lebusa, Mamello Lepitla</t>
+  </si>
+  <si>
+    <t>Parents could not delete an application because the tables have no cascading deletes and RLS blocked it.</t>
+  </si>
+  <si>
+    <t>Deletion was impossible from the app.</t>
+  </si>
+  <si>
+    <t>Created a database function that removes all related records in one transaction, plus storage delete policies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paballo Lebusa </t>
+  </si>
+  <si>
+    <t>28 September 2026 - 25 October 2026</t>
+  </si>
+  <si>
+    <t>Flutter parent app, ASP.NET staff app, Supabase schema and policies, payment proof and verification, confirmation letters, delete application, test data and demonstration.</t>
+  </si>
+  <si>
+    <t>Flutter parent app, ASP.NET staff app And supabase development and integration</t>
+  </si>
+  <si>
+    <t>The most important lesson from Phase 3 was that security rules must be designed together with the features, not added afterwards. Almost every problem we met came from row-level security and storage policies in Supabase rather than from the screens. Features such as deleting an application touch many related tables and uploaded files, so they needed careful ordering and a database function instead of simple queries.</t>
+  </si>
+  <si>
+    <t>The work went well because the Phase 2 designs carried straight into development. The stakeholder’s request for brown and white colours, and for a payment step showing the fee, banking details and payment reference, was built into the Flutter parent app and the ASP.NET staff app. A shared Supabase backend gave both applications the same data, which made integration and testing easier.</t>
+  </si>
+  <si>
+    <t>The hardest parts were the access policies and the features that affect many records at once. Parents and staff need different permissions, and several screens and uploads failed until we corrected the policies. We learned to test each feature with both roles before calling it finished.</t>
+  </si>
+  <si>
+    <t>Tasks were divided according to each member’s strengths, with some members focusing on the parent app, others on the staff app and backend, and others on documentation, testing and project tracking. Contribution was not completely even, and some members had to take on extra work to keep deliverables on schedule. We recorded this in the contribution record..</t>
+  </si>
+  <si>
+    <t>We handled delays by redistributing work and following up through messages, and we had no major conflicts..</t>
+  </si>
+  <si>
+    <t>From the stakeholder we learned that the school wants a simple, clear process that replaces the slow paper-based enrolment, and that payment details must be visible to parents before they upload proof of payment.</t>
+  </si>
+  <si>
+    <t>Staff and payment features, project tracking</t>
+  </si>
+  <si>
+    <t>Parent app development</t>
+  </si>
+  <si>
+    <t>ASP.NET payment verification</t>
+  </si>
+  <si>
+    <t>Unit4/Phase 3</t>
+  </si>
+  <si>
+    <t>WhatsApp</t>
+  </si>
+  <si>
+    <t>Confirmation of the developed system</t>
+  </si>
+  <si>
+    <t>Maleshoane Gweneth Adegbola)–  Principal, Phehello Secondary School</t>
+  </si>
+  <si>
+    <t>Confirmation form sent and signed form received on the same day.</t>
+  </si>
+  <si>
+    <t>Insert the signed form in the SRS, Part E (Figure 4.72).</t>
+  </si>
+  <si>
+    <t>SRS Part E, Figure 4.79</t>
+  </si>
+  <si>
+    <t>Unit 4/Phase 3</t>
+  </si>
+  <si>
+    <t>A member’s GitHub account was left signed in on a school lab computer, so a commit made from that computer showed that member’s name and the author could not be changed.</t>
+  </si>
+  <si>
+    <t>Commits were attributed to the wrong person, which could misrepresent who did the work.</t>
+  </si>
+  <si>
+    <t>Each member committed from their own GitHub account instead, so every contribution is recorded under the right name.</t>
+  </si>
+  <si>
+    <t>1.15</t>
+  </si>
+  <si>
+    <t>1.16</t>
+  </si>
+  <si>
+    <t>1.17</t>
+  </si>
+  <si>
+    <t>1.18</t>
+  </si>
+  <si>
+    <t>1.19</t>
+  </si>
+  <si>
+    <t>1.21</t>
+  </si>
+  <si>
+    <t>1.22</t>
+  </si>
+  <si>
+    <t>1.23</t>
+  </si>
+  <si>
+    <t>1.24</t>
+  </si>
+  <si>
+    <t>1.25</t>
+  </si>
+  <si>
+    <t>1.27</t>
+  </si>
+  <si>
+    <t>1.28</t>
+  </si>
+  <si>
+    <t>1.29</t>
+  </si>
+  <si>
+    <t>Lerato Mahlatsi,Mamello Lepitla, Paballo Lebusa</t>
+  </si>
+  <si>
+    <t>Paballo Lebusa,Mamello Lepitla, Lerato Mahlatsi</t>
+  </si>
+  <si>
+    <t>1.30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microsoft Project Schedule </t>
+  </si>
+  <si>
+    <t>Update the Microsoft Project Schedule for Phase 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Progress Tracker </t>
+  </si>
+  <si>
+    <t>Update the Progress Tracker</t>
+  </si>
+  <si>
+    <t>Github documentation</t>
+  </si>
+  <si>
+    <t>SRS</t>
+  </si>
+  <si>
+    <t>Updated the SRS(Part E)</t>
+  </si>
+  <si>
+    <t>1.20</t>
+  </si>
+  <si>
+    <t>1.31</t>
+  </si>
+  <si>
+    <t>Supabase scheme and security policies</t>
+  </si>
+  <si>
+    <t>1.32</t>
+  </si>
+  <si>
+    <t>Developed parent registration, login, the six-step enrolment wizard and document upload</t>
+  </si>
+  <si>
+    <t>Katleho Makhoali, Mpho Motaung, David Adegbola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flutter : registration, login and enrolment </t>
+  </si>
+  <si>
+    <t>1.33</t>
+  </si>
+  <si>
+    <t>Flutter: payment information and proof of payment</t>
+  </si>
+  <si>
+    <t>Implemented the payment information screen an dproof-of-payment upolad with payment reference</t>
+  </si>
+  <si>
+    <t>Implemented the database scheme, row-level security, storage policies and staff access policies for both apps.</t>
+  </si>
+  <si>
+    <t>1.34</t>
+  </si>
+  <si>
+    <t>Flutter: status, notifications, profile and help</t>
+  </si>
+  <si>
+    <t>Built My Applications, Application Details, Messages and Notifications, Profile and Help &amp; Support</t>
+  </si>
+  <si>
+    <t>1.35</t>
+  </si>
+  <si>
+    <t>ASP.NET: login, dashboards and application lists</t>
+  </si>
+  <si>
+    <t>Developed staff login with role-based access, both dashboards and the application lists</t>
+  </si>
+  <si>
+    <t>Mamello Lepitla, Paballo Lebusa, Lerato Mahlatsi</t>
+  </si>
+  <si>
+    <t>Developed the review page with approve, reject, request corrections and internal notes</t>
+  </si>
+  <si>
+    <t>1.36</t>
+  </si>
+  <si>
+    <t>1.37</t>
+  </si>
+  <si>
+    <t>ASP.NET: payment verification</t>
+  </si>
+  <si>
+    <t>Developed clerk payment verification against the school payment records</t>
+  </si>
+  <si>
+    <t>1.38</t>
+  </si>
+  <si>
+    <t>1.39</t>
+  </si>
+  <si>
+    <t>1.40</t>
+  </si>
+  <si>
+    <t>1.41</t>
+  </si>
+  <si>
+    <t>1.42</t>
+  </si>
+  <si>
+    <t>1.43</t>
+  </si>
+  <si>
+    <t>1.44</t>
+  </si>
+  <si>
+    <t>1.45</t>
+  </si>
+  <si>
+    <t>1.46</t>
+  </si>
+  <si>
+    <t>1.47</t>
+  </si>
+  <si>
+    <t>ASP.NET: messaging and reminders</t>
+  </si>
+  <si>
+    <t>Built the Message Parent and Send Deadline Reminder pages</t>
+  </si>
+  <si>
+    <t>Implemented confirmation letter generation</t>
+  </si>
+  <si>
+    <t>Mamello Lepitla, Paballo Lebusa</t>
+  </si>
+  <si>
+    <t>Implemented parent deletion of an application with related records and files; Paballo wrote the database function</t>
+  </si>
+  <si>
+    <t>Katleho Makhoali, Mpho Motaung, David Adegbola, Paballo Lebusa</t>
+  </si>
+  <si>
+    <t>Prepared fictional learners, sample documents and school payment records</t>
+  </si>
+  <si>
+    <t>Commit code to Github</t>
+  </si>
+  <si>
+    <t>Committed the Flutter and ASP.NET code. Each member committed from their own account after a lab-computer login problem</t>
+  </si>
+  <si>
+    <t>Tested the full flow from parent submission to staff review and payment verification, including role access tests</t>
+  </si>
+  <si>
+    <t>Corrections after lecturer feedback</t>
+  </si>
+  <si>
+    <t>Clearer dashboard charts and a Save &amp; Close button on the enrolment form</t>
+  </si>
+  <si>
+    <t>Stakeholder confirmation of the developed system</t>
+  </si>
+  <si>
+    <t>Sent the confirmation form to the stakeholder and received it signed the same day</t>
+  </si>
+  <si>
+    <t>Final GitHub release, MS Project report and group reflection</t>
+  </si>
+  <si>
+    <t>Final repository release and final project report</t>
+  </si>
+  <si>
+    <t>Final presentation and defence (Assessment 3)</t>
+  </si>
+  <si>
+    <t>Present and defend the system</t>
+  </si>
+  <si>
+    <t>Supabase backend, ASP.NET staff features, test data, SRS</t>
+  </si>
+  <si>
+    <t>Backend security, payment and staff features, documentation</t>
+  </si>
+  <si>
+    <t>Implemented the Supabase schema, row-level security and storage policies. Worked on the payment information and proof-of-payment screens, the ASP.NET staff screens, application review and notes, and confirmation letters. Prepared the test data and updated the SRS (Part E). Took part in integration testing and committed work from her own GitHub account.</t>
+  </si>
+  <si>
+    <t>Staff features, database fixes, Project schedule and tracker</t>
+  </si>
+  <si>
+    <t>Worked on the ASP.NET staff screens, application review, confirmation letters and the payment screens. Wrote the staff access patch with Mamello and the database function for deleting applications. Updated the Microsoft Project schedule and the Progress Tracker. Took part in integration testing and committed from his own GitHub account.</t>
+  </si>
+  <si>
+    <t>Flutter parent app, GitHub</t>
+  </si>
+  <si>
+    <t>Parent app development, GitHub documentation</t>
+  </si>
+  <si>
+    <t>Developed the Flutter registration, login, enrolment and status screens and the delete-application feature with Mpho and David. Wrote the GitHub documentation. Took part in integration testing and committed from his own GitHub account.</t>
+  </si>
+  <si>
+    <t>Financial Clerk features</t>
+  </si>
+  <si>
+    <t>Developed the clerk payment verification against the school payment records and worked on the ASP.NET staff screens. Took part in integration testing and committed from her own GitHub account.</t>
+  </si>
+  <si>
+    <t>Flutter parent app, stakeholder communication</t>
+  </si>
+  <si>
+    <t>Parent app development, stakeholder coordination</t>
+  </si>
+  <si>
+    <t>Developed the Flutter enrolment screens and the delete-application feature with Katleho and Mpho. Contacted the stakeholder, sent the confirmation form and received the signed form on 25 Oct 2026. Took part in integration testing and committed from his own GitHub account.</t>
+  </si>
+  <si>
+    <t>Developed the Flutter enrolment, status and notification screens and the delete-application feature with Katleho and David. Took part in integration testing and committed from his own GitHub account.</t>
+  </si>
+  <si>
+    <t>Flutter parent app</t>
   </si>
 </sst>
 </file>
@@ -1096,7 +1423,7 @@
     <numFmt numFmtId="166" formatCode="0&quot;%&quot;"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1132,6 +1459,12 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -1237,7 +1570,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1344,6 +1677,11 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1518,7 +1856,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>25</c:v>
+                  <c:v>46</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1672,7 +2010,7 @@
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
   <global>
     <keyFlags>
       <key name="_Self">
@@ -1756,7 +2094,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TaskProgressTable" displayName="TaskProgressTable" ref="A2:M101">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TaskProgressTable" displayName="TaskProgressTable" ref="A2:M90">
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Task ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Reporting Phase"/>
@@ -2227,8 +2565,8 @@
         <v>46</v>
       </c>
       <c r="G4" s="10">
-        <f>COUNTIF('Task Progress'!H2:H101,"Completed")</f>
-        <v>25</v>
+        <f>COUNTIF('Task Progress'!H2:H90,"Completed")</f>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="27.95" customHeight="1">
@@ -2242,7 +2580,7 @@
         <v>48</v>
       </c>
       <c r="G5" s="10">
-        <f>COUNTIF('Task Progress'!H2:H101,"In Progress")</f>
+        <f>COUNTIF('Task Progress'!H2:H90,"In Progress")</f>
         <v>0</v>
       </c>
     </row>
@@ -2257,7 +2595,7 @@
         <v>50</v>
       </c>
       <c r="G6" s="10">
-        <f>COUNTIF('Task Progress'!H2:H101,"Not Started")</f>
+        <f>COUNTIF('Task Progress'!H2:H90,"Not Started")</f>
         <v>0</v>
       </c>
     </row>
@@ -2272,7 +2610,7 @@
         <v>52</v>
       </c>
       <c r="G7" s="10">
-        <f>COUNTIF('Task Progress'!H2:H101,"Delayed")</f>
+        <f>COUNTIF('Task Progress'!H2:H90,"Delayed")</f>
         <v>0</v>
       </c>
     </row>
@@ -2281,13 +2619,13 @@
         <v>53</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>256</v>
+        <v>308</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G8" s="10">
-        <f>COUNTIF('Task Progress'!H2:H101,"Blocked")</f>
+        <f>COUNTIF('Task Progress'!H2:H90,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
@@ -2296,13 +2634,13 @@
         <v>55</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>290</v>
+        <v>309</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>56</v>
       </c>
       <c r="G9" s="11">
-        <f ca="1">COUNTIF('Task Progress'!M2:M101,"Overdue")</f>
+        <f ca="1">COUNTIF('Task Progress'!M2:M90,"Overdue")</f>
         <v>0</v>
       </c>
     </row>
@@ -2333,14 +2671,14 @@
         <v>60</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>291</v>
+        <v>310</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>61</v>
       </c>
       <c r="G12" s="10">
         <f>COUNTIF('Individual Contributions'!E3:E201,"?*")</f>
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="48" customHeight="1">
@@ -2348,14 +2686,14 @@
         <v>62</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>63</v>
       </c>
       <c r="G13" s="10">
         <f>COUNTIFS('Individual Contributions'!E3:E201,"?*",'Individual Contributions'!J3:J201,"Yes")</f>
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="48" customHeight="1">
@@ -2363,7 +2701,7 @@
         <v>64</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>65</v>
@@ -2379,7 +2717,7 @@
       </c>
       <c r="G15" s="11">
         <f>COUNT('Stakeholder Engagement'!A3:A101)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2402,7 +2740,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:M101"/>
+  <dimension ref="A1:M90"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2479,19 +2817,19 @@
     </row>
     <row r="3" spans="1:13" ht="57">
       <c r="A3" s="16" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C3" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="E3" s="12" t="s">
         <v>187</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>211</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="F3" s="13">
         <v>46251</v>
@@ -2511,22 +2849,22 @@
       </c>
       <c r="L3" s="12"/>
       <c r="M3" s="17" t="str">
-        <f t="shared" ref="M3:M34" ca="1" si="0">IF(D3="","",IF(H3="Completed","Completed",IF(H3="Blocked","Blocked",IF(H3="Delayed","Delayed",IF(AND(G3&lt;&gt;"",G3&lt;TODAY(),H3&lt;&gt;"Completed"),"Overdue","On Track")))))</f>
+        <f t="shared" ref="M3:M27" ca="1" si="0">IF(D3="","",IF(H3="Completed","Completed",IF(H3="Blocked","Blocked",IF(H3="Delayed","Delayed",IF(AND(G3&lt;&gt;"",G3&lt;TODAY(),H3&lt;&gt;"Completed"),"Overdue","On Track")))))</f>
         <v>Completed</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="57">
       <c r="A4" s="16" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>152</v>
@@ -2555,16 +2893,16 @@
     </row>
     <row r="5" spans="1:13" ht="57">
       <c r="A5" s="16" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>151</v>
@@ -2593,19 +2931,19 @@
     </row>
     <row r="6" spans="1:13" ht="57">
       <c r="A6" s="16" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F6" s="13">
         <v>46258</v>
@@ -2631,16 +2969,16 @@
     </row>
     <row r="7" spans="1:13" ht="57">
       <c r="A7" s="16" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>151</v>
@@ -2669,16 +3007,16 @@
     </row>
     <row r="8" spans="1:13" ht="42.75">
       <c r="A8" s="16" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>153</v>
@@ -2707,16 +3045,16 @@
     </row>
     <row r="9" spans="1:13" ht="28.5">
       <c r="A9" s="16" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E9" s="12" t="s">
         <v>151</v>
@@ -2745,16 +3083,16 @@
     </row>
     <row r="10" spans="1:13" ht="42.75">
       <c r="A10" s="16" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E10" s="12" t="s">
         <v>153</v>
@@ -2783,19 +3121,19 @@
     </row>
     <row r="11" spans="1:13" ht="42.75">
       <c r="A11" s="16" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F11" s="13">
         <v>46258</v>
@@ -2821,19 +3159,19 @@
     </row>
     <row r="12" spans="1:13" ht="42.75">
       <c r="A12" s="16" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D12" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="E12" s="12" t="s">
         <v>221</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>219</v>
       </c>
       <c r="F12" s="13">
         <v>46258</v>
@@ -2859,16 +3197,16 @@
     </row>
     <row r="13" spans="1:13" ht="42.75">
       <c r="A13" s="16" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E13" s="12" t="s">
         <v>152</v>
@@ -2897,16 +3235,16 @@
     </row>
     <row r="14" spans="1:13" ht="42.75">
       <c r="A14" s="16" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B14" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E14" s="12" t="s">
         <v>151</v>
@@ -2935,16 +3273,16 @@
     </row>
     <row r="15" spans="1:13" ht="42.75">
       <c r="A15" s="16" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E15" s="12" t="s">
         <v>152</v>
@@ -2973,19 +3311,19 @@
     </row>
     <row r="16" spans="1:13" ht="28.5">
       <c r="A16" s="16" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F16" s="13">
         <v>46265</v>
@@ -3010,17 +3348,17 @@
       </c>
     </row>
     <row r="17" spans="1:13" ht="42.75">
-      <c r="A17" s="16">
-        <v>1.1499999999999999</v>
+      <c r="A17" s="16" t="s">
+        <v>348</v>
       </c>
       <c r="B17" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="D17" s="12" t="s">
         <v>256</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>254</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>255</v>
       </c>
       <c r="E17" s="12" t="s">
         <v>152</v>
@@ -3048,17 +3386,17 @@
       </c>
     </row>
     <row r="18" spans="1:13" ht="28.5">
-      <c r="A18" s="16">
-        <v>1.1599999999999999</v>
+      <c r="A18" s="16" t="s">
+        <v>349</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E18" s="12" t="s">
         <v>153</v>
@@ -3086,20 +3424,20 @@
       </c>
     </row>
     <row r="19" spans="1:13" ht="28.5">
-      <c r="A19" s="16">
-        <v>1.17</v>
+      <c r="A19" s="16" t="s">
+        <v>350</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F19" s="13">
         <v>46274</v>
@@ -3124,17 +3462,17 @@
       </c>
     </row>
     <row r="20" spans="1:13" ht="42.75">
-      <c r="A20" s="16">
-        <v>1.18</v>
+      <c r="A20" s="16" t="s">
+        <v>351</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E20" s="12" t="s">
         <v>151</v>
@@ -3162,20 +3500,20 @@
       </c>
     </row>
     <row r="21" spans="1:13" ht="28.5">
-      <c r="A21" s="16">
-        <v>1.19</v>
+      <c r="A21" s="16" t="s">
+        <v>352</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>292</v>
+        <v>361</v>
       </c>
       <c r="F21" s="13">
         <v>46277</v>
@@ -3200,20 +3538,20 @@
       </c>
     </row>
     <row r="22" spans="1:13" ht="28.5">
-      <c r="A22" s="16">
-        <v>1.2</v>
+      <c r="A22" s="16" t="s">
+        <v>371</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>292</v>
+        <v>361</v>
       </c>
       <c r="F22" s="13">
         <v>46281</v>
@@ -3238,20 +3576,20 @@
       </c>
     </row>
     <row r="23" spans="1:13" ht="28.5">
-      <c r="A23" s="16">
-        <v>1.21</v>
+      <c r="A23" s="16" t="s">
+        <v>353</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F23" s="13">
         <v>46279</v>
@@ -3276,17 +3614,17 @@
       </c>
     </row>
     <row r="24" spans="1:13">
-      <c r="A24" s="16">
-        <v>1.22</v>
+      <c r="A24" s="16" t="s">
+        <v>354</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E24" s="12" t="s">
         <v>152</v>
@@ -3314,17 +3652,17 @@
       </c>
     </row>
     <row r="25" spans="1:13">
-      <c r="A25" s="16">
-        <v>1.23</v>
+      <c r="A25" s="16" t="s">
+        <v>355</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E25" s="12" t="s">
         <v>153</v>
@@ -3352,20 +3690,20 @@
       </c>
     </row>
     <row r="26" spans="1:13" ht="28.5">
-      <c r="A26" s="16">
-        <v>1.24</v>
+      <c r="A26" s="16" t="s">
+        <v>356</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>152</v>
+        <v>362</v>
       </c>
       <c r="F26" s="13">
         <v>46279</v>
@@ -3390,17 +3728,17 @@
       </c>
     </row>
     <row r="27" spans="1:13">
-      <c r="A27" s="16">
-        <v>1.25</v>
+      <c r="A27" s="16" t="s">
+        <v>357</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E27" s="12" t="s">
         <v>151</v>
@@ -3427,382 +3765,802 @@
         <v>Completed</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
-      <c r="A28" s="16"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="13"/>
-      <c r="H28" s="12"/>
-      <c r="I28" s="14"/>
+    <row r="28" spans="1:13" ht="28.5">
+      <c r="A28" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>364</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="F28" s="13">
+        <v>46297</v>
+      </c>
+      <c r="G28" s="13">
+        <v>46318</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I28" s="14">
+        <v>100</v>
+      </c>
       <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
+      <c r="K28" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L28" s="12"/>
       <c r="M28" s="17" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:13">
-      <c r="A29" s="16"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="12"/>
-      <c r="I29" s="14"/>
+        <f t="shared" ref="M28:M55" ca="1" si="1">IF(D28="","",IF(H28="Completed","Completed",IF(H28="Blocked","Blocked",IF(H28="Delayed","Delayed",IF(AND(G28&lt;&gt;"",G28&lt;TODAY(),H28&lt;&gt;"Completed"),"Overdue","On Track")))))</f>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="28.5">
+      <c r="A29" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>320</v>
+      </c>
+      <c r="F29" s="13">
+        <v>46297</v>
+      </c>
+      <c r="G29" s="13">
+        <v>46318</v>
+      </c>
+      <c r="H29" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I29" s="14">
+        <v>100</v>
+      </c>
       <c r="J29" s="12"/>
-      <c r="K29" s="12"/>
+      <c r="K29" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L29" s="12"/>
       <c r="M29" s="17" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v/>
+        <f t="shared" ca="1" si="1"/>
+        <v>Completed</v>
       </c>
     </row>
     <row r="30" spans="1:13">
-      <c r="A30" s="16"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="12"/>
-      <c r="I30" s="14"/>
+      <c r="A30" s="16" t="s">
+        <v>360</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F30" s="13">
+        <v>46297</v>
+      </c>
+      <c r="G30" s="13">
+        <v>46318</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I30" s="14">
+        <v>100</v>
+      </c>
       <c r="J30" s="12"/>
-      <c r="K30" s="12"/>
+      <c r="K30" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L30" s="12"/>
       <c r="M30" s="17" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v/>
+        <f t="shared" ca="1" si="1"/>
+        <v>Completed</v>
       </c>
     </row>
     <row r="31" spans="1:13">
-      <c r="A31" s="16"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="12"/>
-      <c r="I31" s="14"/>
+      <c r="A31" s="16" t="s">
+        <v>363</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="F31" s="13">
+        <v>46297</v>
+      </c>
+      <c r="G31" s="13">
+        <v>46320</v>
+      </c>
+      <c r="H31" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I31" s="14">
+        <v>100</v>
+      </c>
       <c r="J31" s="12"/>
-      <c r="K31" s="12"/>
+      <c r="K31" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L31" s="12"/>
       <c r="M31" s="17" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:13">
-      <c r="A32" s="16"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="12"/>
-      <c r="I32" s="14"/>
+        <f t="shared" ca="1" si="1"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" ht="42.75">
+      <c r="A32" s="16" t="s">
+        <v>372</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>381</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="F32" s="40">
+        <v>46297</v>
+      </c>
+      <c r="G32" s="40">
+        <v>46301</v>
+      </c>
+      <c r="H32" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I32" s="14">
+        <v>100</v>
+      </c>
       <c r="J32" s="12"/>
-      <c r="K32" s="12"/>
+      <c r="K32" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L32" s="12"/>
       <c r="M32" s="17" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="1:13">
-      <c r="A33" s="16"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="12"/>
-      <c r="I33" s="14"/>
+        <f t="shared" ca="1" si="1"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" ht="28.5">
+      <c r="A33" s="16" t="s">
+        <v>374</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C33" t="s">
+        <v>377</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>376</v>
+      </c>
+      <c r="F33" s="13">
+        <v>46301</v>
+      </c>
+      <c r="G33" s="13">
+        <v>46307</v>
+      </c>
+      <c r="H33" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I33" s="14">
+        <v>100</v>
+      </c>
       <c r="J33" s="12"/>
-      <c r="K33" s="12"/>
+      <c r="K33" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L33" s="12"/>
       <c r="M33" s="17" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="1:13">
-      <c r="A34" s="16"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="14"/>
+        <f t="shared" ca="1" si="1"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" ht="42.75">
+      <c r="A34" s="16" t="s">
+        <v>378</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>379</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>380</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>376</v>
+      </c>
+      <c r="F34" s="13">
+        <v>46307</v>
+      </c>
+      <c r="G34" s="13">
+        <v>46311</v>
+      </c>
+      <c r="H34" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I34" s="14">
+        <v>100</v>
+      </c>
       <c r="J34" s="12"/>
-      <c r="K34" s="12"/>
+      <c r="K34" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L34" s="12"/>
       <c r="M34" s="17" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="1:13">
-      <c r="A35" s="16"/>
-      <c r="B35" s="12"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="12"/>
-      <c r="I35" s="14"/>
+        <f t="shared" ca="1" si="1"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" ht="42.75">
+      <c r="A35" s="16" t="s">
+        <v>382</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>383</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>376</v>
+      </c>
+      <c r="F35" s="13">
+        <v>46308</v>
+      </c>
+      <c r="G35" s="13">
+        <v>46312</v>
+      </c>
+      <c r="H35" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I35" s="14">
+        <v>100</v>
+      </c>
       <c r="J35" s="12"/>
-      <c r="K35" s="12"/>
+      <c r="K35" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L35" s="12"/>
       <c r="M35" s="17" t="str">
-        <f t="shared" ref="M35:M66" ca="1" si="1">IF(D35="","",IF(H35="Completed","Completed",IF(H35="Blocked","Blocked",IF(H35="Delayed","Delayed",IF(AND(G35&lt;&gt;"",G35&lt;TODAY(),H35&lt;&gt;"Completed"),"Overdue","On Track")))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="1:13">
-      <c r="A36" s="16"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
-      <c r="H36" s="12"/>
-      <c r="I36" s="14"/>
+        <f t="shared" ca="1" si="1"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" ht="42.75">
+      <c r="A36" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="F36" s="13">
+        <v>46307</v>
+      </c>
+      <c r="G36" s="13">
+        <v>46321</v>
+      </c>
+      <c r="H36" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I36" s="14">
+        <v>100</v>
+      </c>
       <c r="J36" s="12"/>
-      <c r="K36" s="12"/>
+      <c r="K36" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L36" s="12"/>
       <c r="M36" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="1:13">
-      <c r="A37" s="16"/>
-      <c r="B37" s="12"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="13"/>
-      <c r="H37" s="12"/>
-      <c r="I37" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" ht="42.75">
+      <c r="A37" s="16" t="s">
+        <v>390</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="F37" s="13">
+        <v>46308</v>
+      </c>
+      <c r="G37" s="13">
+        <v>46310</v>
+      </c>
+      <c r="H37" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I37" s="14">
+        <v>100</v>
+      </c>
       <c r="J37" s="12"/>
-      <c r="K37" s="12"/>
+      <c r="K37" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L37" s="12"/>
       <c r="M37" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="1:13">
-      <c r="A38" s="16"/>
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="12"/>
-      <c r="I38" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" ht="42.75">
+      <c r="A38" s="16" t="s">
+        <v>391</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>392</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="F38" s="13">
+        <v>46307</v>
+      </c>
+      <c r="G38" s="13">
+        <v>46311</v>
+      </c>
+      <c r="H38" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I38" s="14">
+        <v>100</v>
+      </c>
       <c r="J38" s="12"/>
-      <c r="K38" s="12"/>
+      <c r="K38" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L38" s="12"/>
       <c r="M38" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="1:13">
-      <c r="A39" s="16"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="13"/>
-      <c r="H39" s="12"/>
-      <c r="I39" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" ht="42.75">
+      <c r="A39" s="16" t="s">
+        <v>394</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>404</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>405</v>
+      </c>
+      <c r="E39" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="F39" s="13">
+        <v>46308</v>
+      </c>
+      <c r="G39" s="13">
+        <v>46311</v>
+      </c>
+      <c r="H39" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I39" s="14">
+        <v>100</v>
+      </c>
       <c r="J39" s="12"/>
-      <c r="K39" s="12"/>
+      <c r="K39" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L39" s="12"/>
       <c r="M39" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="1:13">
-      <c r="A40" s="16"/>
-      <c r="B40" s="12"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" ht="28.5">
+      <c r="A40" s="16" t="s">
+        <v>395</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>313</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="E40" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="F40" s="13">
+        <v>46308</v>
+      </c>
+      <c r="G40" s="13">
+        <v>46313</v>
+      </c>
+      <c r="H40" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I40" s="14">
+        <v>100</v>
+      </c>
       <c r="J40" s="12"/>
-      <c r="K40" s="12"/>
+      <c r="K40" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L40" s="12"/>
       <c r="M40" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="1:13">
-      <c r="A41" s="16"/>
-      <c r="B41" s="12"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="12"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="13"/>
-      <c r="H41" s="12"/>
-      <c r="I41" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" ht="42.75">
+      <c r="A41" s="16" t="s">
+        <v>396</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>408</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>409</v>
+      </c>
+      <c r="F41" s="13">
+        <v>46308</v>
+      </c>
+      <c r="G41" s="13">
+        <v>46313</v>
+      </c>
+      <c r="H41" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I41" s="14">
+        <v>100</v>
+      </c>
       <c r="J41" s="12"/>
-      <c r="K41" s="12"/>
+      <c r="K41" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L41" s="12"/>
       <c r="M41" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="1:13">
-      <c r="A42" s="16"/>
-      <c r="B42" s="12"/>
-      <c r="C42" s="12"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="12"/>
-      <c r="F42" s="13"/>
-      <c r="G42" s="13"/>
-      <c r="H42" s="12"/>
-      <c r="I42" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" ht="42.75">
+      <c r="A42" s="16" t="s">
+        <v>397</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>410</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="F42" s="13">
+        <v>46314</v>
+      </c>
+      <c r="G42" s="13">
+        <v>46314</v>
+      </c>
+      <c r="H42" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I42" s="14">
+        <v>100</v>
+      </c>
       <c r="J42" s="12"/>
-      <c r="K42" s="12"/>
+      <c r="K42" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L42" s="12"/>
       <c r="M42" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="1:13">
-      <c r="A43" s="16"/>
-      <c r="B43" s="12"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="12"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="13"/>
-      <c r="H43" s="12"/>
-      <c r="I43" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" ht="42.75">
+      <c r="A43" s="16" t="s">
+        <v>398</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>411</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>412</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="F43" s="13">
+        <v>46314</v>
+      </c>
+      <c r="G43" s="13">
+        <v>46316</v>
+      </c>
+      <c r="H43" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I43" s="14">
+        <v>100</v>
+      </c>
       <c r="J43" s="12"/>
-      <c r="K43" s="12"/>
+      <c r="K43" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L43" s="12"/>
       <c r="M43" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="1:13">
-      <c r="A44" s="16"/>
-      <c r="B44" s="12"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="12"/>
-      <c r="F44" s="13"/>
-      <c r="G44" s="13"/>
-      <c r="H44" s="12"/>
-      <c r="I44" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" ht="42.75">
+      <c r="A44" s="16" t="s">
+        <v>399</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>316</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>413</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="F44" s="13">
+        <v>46314</v>
+      </c>
+      <c r="G44" s="13">
+        <v>46318</v>
+      </c>
+      <c r="H44" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I44" s="14">
+        <v>100</v>
+      </c>
       <c r="J44" s="12"/>
-      <c r="K44" s="12"/>
+      <c r="K44" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L44" s="12"/>
       <c r="M44" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="1:13">
-      <c r="A45" s="16"/>
-      <c r="B45" s="12"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="13"/>
-      <c r="G45" s="13"/>
-      <c r="H45" s="12"/>
-      <c r="I45" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" ht="28.5">
+      <c r="A45" s="16" t="s">
+        <v>400</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>414</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>415</v>
+      </c>
+      <c r="E45" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="F45" s="13">
+        <v>46315</v>
+      </c>
+      <c r="G45" s="13">
+        <v>46318</v>
+      </c>
+      <c r="H45" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I45" s="14">
+        <v>100</v>
+      </c>
       <c r="J45" s="12"/>
-      <c r="K45" s="12"/>
+      <c r="K45" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L45" s="12"/>
       <c r="M45" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="1:13">
-      <c r="A46" s="16"/>
-      <c r="B46" s="12"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="12"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="13"/>
-      <c r="H46" s="12"/>
-      <c r="I46" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" ht="57">
+      <c r="A46" s="16" t="s">
+        <v>401</v>
+      </c>
+      <c r="B46" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>416</v>
+      </c>
+      <c r="D46" s="12" t="s">
+        <v>417</v>
+      </c>
+      <c r="E46" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="F46" s="13">
+        <v>46318</v>
+      </c>
+      <c r="G46" s="13">
+        <v>46320</v>
+      </c>
+      <c r="H46" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I46" s="14">
+        <v>100</v>
+      </c>
       <c r="J46" s="12"/>
-      <c r="K46" s="12"/>
+      <c r="K46" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L46" s="12"/>
       <c r="M46" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="47" spans="1:13">
-      <c r="A47" s="16"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="13"/>
-      <c r="H47" s="12"/>
-      <c r="I47" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" ht="71.25">
+      <c r="A47" s="16" t="s">
+        <v>402</v>
+      </c>
+      <c r="B47" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>418</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>419</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F47" s="13">
+        <v>46314</v>
+      </c>
+      <c r="G47" s="13">
+        <v>46318</v>
+      </c>
+      <c r="H47" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I47" s="14">
+        <v>100</v>
+      </c>
       <c r="J47" s="12"/>
-      <c r="K47" s="12"/>
+      <c r="K47" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L47" s="12"/>
       <c r="M47" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="1:13">
-      <c r="A48" s="16"/>
-      <c r="B48" s="12"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
-      <c r="H48" s="12"/>
-      <c r="I48" s="14"/>
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" ht="57">
+      <c r="A48" s="16" t="s">
+        <v>403</v>
+      </c>
+      <c r="B48" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>420</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>421</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="F48" s="13">
+        <v>46321</v>
+      </c>
+      <c r="G48" s="13">
+        <v>46323</v>
+      </c>
+      <c r="H48" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I48" s="14">
+        <v>100</v>
+      </c>
       <c r="J48" s="12"/>
-      <c r="K48" s="12"/>
+      <c r="K48" s="12" t="s">
+        <v>154</v>
+      </c>
       <c r="L48" s="12"/>
       <c r="M48" s="17" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
+        <v>Completed</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -3945,7 +4703,7 @@
       <c r="K56" s="12"/>
       <c r="L56" s="12"/>
       <c r="M56" s="17" t="str">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ref="M56:M90" ca="1" si="2">IF(D56="","",IF(H56="Completed","Completed",IF(H56="Blocked","Blocked",IF(H56="Delayed","Delayed",IF(AND(G56&lt;&gt;"",G56&lt;TODAY(),H56&lt;&gt;"Completed"),"Overdue","On Track")))))</f>
         <v/>
       </c>
     </row>
@@ -3963,7 +4721,7 @@
       <c r="K57" s="12"/>
       <c r="L57" s="12"/>
       <c r="M57" s="17" t="str">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
     </row>
@@ -3981,7 +4739,7 @@
       <c r="K58" s="12"/>
       <c r="L58" s="12"/>
       <c r="M58" s="17" t="str">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
     </row>
@@ -3999,7 +4757,7 @@
       <c r="K59" s="12"/>
       <c r="L59" s="12"/>
       <c r="M59" s="17" t="str">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
     </row>
@@ -4017,7 +4775,7 @@
       <c r="K60" s="12"/>
       <c r="L60" s="12"/>
       <c r="M60" s="17" t="str">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
     </row>
@@ -4035,7 +4793,7 @@
       <c r="K61" s="12"/>
       <c r="L61" s="12"/>
       <c r="M61" s="17" t="str">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
     </row>
@@ -4053,7 +4811,7 @@
       <c r="K62" s="12"/>
       <c r="L62" s="12"/>
       <c r="M62" s="17" t="str">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
     </row>
@@ -4071,7 +4829,7 @@
       <c r="K63" s="12"/>
       <c r="L63" s="12"/>
       <c r="M63" s="17" t="str">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
     </row>
@@ -4089,7 +4847,7 @@
       <c r="K64" s="12"/>
       <c r="L64" s="12"/>
       <c r="M64" s="17" t="str">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
     </row>
@@ -4107,7 +4865,7 @@
       <c r="K65" s="12"/>
       <c r="L65" s="12"/>
       <c r="M65" s="17" t="str">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
     </row>
@@ -4125,7 +4883,7 @@
       <c r="K66" s="12"/>
       <c r="L66" s="12"/>
       <c r="M66" s="17" t="str">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
     </row>
@@ -4143,7 +4901,7 @@
       <c r="K67" s="12"/>
       <c r="L67" s="12"/>
       <c r="M67" s="17" t="str">
-        <f t="shared" ref="M67:M101" ca="1" si="2">IF(D67="","",IF(H67="Completed","Completed",IF(H67="Blocked","Blocked",IF(H67="Delayed","Delayed",IF(AND(G67&lt;&gt;"",G67&lt;TODAY(),H67&lt;&gt;"Completed"),"Overdue","On Track")))))</f>
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
     </row>
@@ -4544,217 +5302,19 @@
       </c>
     </row>
     <row r="90" spans="1:13">
-      <c r="A90" s="16"/>
-      <c r="B90" s="12"/>
-      <c r="C90" s="12"/>
-      <c r="D90" s="12"/>
+      <c r="A90" s="18"/>
+      <c r="B90" s="19"/>
+      <c r="C90" s="19"/>
+      <c r="D90" s="19"/>
       <c r="E90" s="12"/>
-      <c r="F90" s="13"/>
-      <c r="G90" s="13"/>
-      <c r="H90" s="12"/>
-      <c r="I90" s="14"/>
-      <c r="J90" s="12"/>
-      <c r="K90" s="12"/>
-      <c r="L90" s="12"/>
-      <c r="M90" s="17" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="91" spans="1:13">
-      <c r="A91" s="16"/>
-      <c r="B91" s="12"/>
-      <c r="C91" s="12"/>
-      <c r="D91" s="12"/>
-      <c r="E91" s="12"/>
-      <c r="F91" s="13"/>
-      <c r="G91" s="13"/>
-      <c r="H91" s="12"/>
-      <c r="I91" s="14"/>
-      <c r="J91" s="12"/>
-      <c r="K91" s="12"/>
-      <c r="L91" s="12"/>
-      <c r="M91" s="17" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="92" spans="1:13">
-      <c r="A92" s="16"/>
-      <c r="B92" s="12"/>
-      <c r="C92" s="12"/>
-      <c r="D92" s="12"/>
-      <c r="E92" s="12"/>
-      <c r="F92" s="13"/>
-      <c r="G92" s="13"/>
-      <c r="H92" s="12"/>
-      <c r="I92" s="14"/>
-      <c r="J92" s="12"/>
-      <c r="K92" s="12"/>
-      <c r="L92" s="12"/>
-      <c r="M92" s="17" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="93" spans="1:13">
-      <c r="A93" s="16"/>
-      <c r="B93" s="12"/>
-      <c r="C93" s="12"/>
-      <c r="D93" s="12"/>
-      <c r="E93" s="12"/>
-      <c r="F93" s="13"/>
-      <c r="G93" s="13"/>
-      <c r="H93" s="12"/>
-      <c r="I93" s="14"/>
-      <c r="J93" s="12"/>
-      <c r="K93" s="12"/>
-      <c r="L93" s="12"/>
-      <c r="M93" s="17" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="94" spans="1:13">
-      <c r="A94" s="16"/>
-      <c r="B94" s="12"/>
-      <c r="C94" s="12"/>
-      <c r="D94" s="12"/>
-      <c r="E94" s="12"/>
-      <c r="F94" s="13"/>
-      <c r="G94" s="13"/>
-      <c r="H94" s="12"/>
-      <c r="I94" s="14"/>
-      <c r="J94" s="12"/>
-      <c r="K94" s="12"/>
-      <c r="L94" s="12"/>
-      <c r="M94" s="17" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="95" spans="1:13">
-      <c r="A95" s="16"/>
-      <c r="B95" s="12"/>
-      <c r="C95" s="12"/>
-      <c r="D95" s="12"/>
-      <c r="E95" s="12"/>
-      <c r="F95" s="13"/>
-      <c r="G95" s="13"/>
-      <c r="H95" s="12"/>
-      <c r="I95" s="14"/>
-      <c r="J95" s="12"/>
-      <c r="K95" s="12"/>
-      <c r="L95" s="12"/>
-      <c r="M95" s="17" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="96" spans="1:13">
-      <c r="A96" s="16"/>
-      <c r="B96" s="12"/>
-      <c r="C96" s="12"/>
-      <c r="D96" s="12"/>
-      <c r="E96" s="12"/>
-      <c r="F96" s="13"/>
-      <c r="G96" s="13"/>
-      <c r="H96" s="12"/>
-      <c r="I96" s="14"/>
-      <c r="J96" s="12"/>
-      <c r="K96" s="12"/>
-      <c r="L96" s="12"/>
-      <c r="M96" s="17" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="97" spans="1:13">
-      <c r="A97" s="16"/>
-      <c r="B97" s="12"/>
-      <c r="C97" s="12"/>
-      <c r="D97" s="12"/>
-      <c r="E97" s="12"/>
-      <c r="F97" s="13"/>
-      <c r="G97" s="13"/>
-      <c r="H97" s="12"/>
-      <c r="I97" s="14"/>
-      <c r="J97" s="12"/>
-      <c r="K97" s="12"/>
-      <c r="L97" s="12"/>
-      <c r="M97" s="17" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="98" spans="1:13">
-      <c r="A98" s="16"/>
-      <c r="B98" s="12"/>
-      <c r="C98" s="12"/>
-      <c r="D98" s="12"/>
-      <c r="E98" s="12"/>
-      <c r="F98" s="13"/>
-      <c r="G98" s="13"/>
-      <c r="H98" s="12"/>
-      <c r="I98" s="14"/>
-      <c r="J98" s="12"/>
-      <c r="K98" s="12"/>
-      <c r="L98" s="12"/>
-      <c r="M98" s="17" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="99" spans="1:13">
-      <c r="A99" s="16"/>
-      <c r="B99" s="12"/>
-      <c r="C99" s="12"/>
-      <c r="D99" s="12"/>
-      <c r="E99" s="12"/>
-      <c r="F99" s="13"/>
-      <c r="G99" s="13"/>
-      <c r="H99" s="12"/>
-      <c r="I99" s="14"/>
-      <c r="J99" s="12"/>
-      <c r="K99" s="12"/>
-      <c r="L99" s="12"/>
-      <c r="M99" s="17" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="100" spans="1:13">
-      <c r="A100" s="16"/>
-      <c r="B100" s="12"/>
-      <c r="C100" s="12"/>
-      <c r="D100" s="12"/>
-      <c r="E100" s="12"/>
-      <c r="F100" s="13"/>
-      <c r="G100" s="13"/>
-      <c r="H100" s="12"/>
-      <c r="I100" s="14"/>
-      <c r="J100" s="12"/>
-      <c r="K100" s="12"/>
-      <c r="L100" s="12"/>
-      <c r="M100" s="17" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="101" spans="1:13">
-      <c r="A101" s="18"/>
-      <c r="B101" s="19"/>
-      <c r="C101" s="19"/>
-      <c r="D101" s="19"/>
-      <c r="E101" s="19"/>
-      <c r="F101" s="20"/>
-      <c r="G101" s="20"/>
-      <c r="H101" s="19"/>
-      <c r="I101" s="21"/>
-      <c r="J101" s="19"/>
-      <c r="K101" s="19"/>
-      <c r="L101" s="19"/>
-      <c r="M101" s="22" t="str">
+      <c r="F90" s="20"/>
+      <c r="G90" s="20"/>
+      <c r="H90" s="19"/>
+      <c r="I90" s="21"/>
+      <c r="J90" s="19"/>
+      <c r="K90" s="19"/>
+      <c r="L90" s="19"/>
+      <c r="M90" s="22" t="str">
         <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
@@ -4763,7 +5323,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:M1"/>
   </mergeCells>
-  <conditionalFormatting sqref="H3:H101">
+  <conditionalFormatting sqref="H3:H90">
     <cfRule type="expression" dxfId="11" priority="1">
       <formula>H3="Completed"</formula>
     </cfRule>
@@ -4777,15 +5337,20 @@
       <formula>H3="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I101">
-    <cfRule type="dataBar" priority="6">
+  <conditionalFormatting sqref="M3:M90">
+    <cfRule type="expression" dxfId="7" priority="5">
+      <formula>M3="Overdue"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3:I90">
+    <cfRule type="dataBar" priority="136">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF1F5A94"/>
       </dataBar>
     </cfRule>
-    <cfRule type="dataBar" priority="7">
+    <cfRule type="dataBar" priority="137">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4798,22 +5363,17 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M3:M101">
-    <cfRule type="expression" dxfId="7" priority="5">
-      <formula>M3="Overdue"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" sqref="B3:B101" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="B3:B90" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Unit 1 / Phase 1,Phase 2,Phase 3,Final"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="H3:H101" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" sqref="H3:H90" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"Not Started,In Progress,Completed,Delayed,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="I3:I101" xr:uid="{00000000-0002-0000-0200-000002000000}">
+    <dataValidation type="list" sqref="I3:I90" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"0,25,50,75,100"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="K3:K101" xr:uid="{00000000-0002-0000-0200-000003000000}">
+    <dataValidation type="list" sqref="K3:K90" xr:uid="{00000000-0002-0000-0200-000003000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4833,7 +5393,7 @@
               <x14:axisColor auto="1"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>I3:I101</xm:sqref>
+          <xm:sqref>I3:I90</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4925,13 +5485,13 @@
         <v>32</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="G3" s="13">
         <v>46265</v>
@@ -4947,7 +5507,7 @@
         <v>46265</v>
       </c>
       <c r="L3" s="17" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="28.5">
@@ -4961,13 +5521,13 @@
         <v>32</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="G4" s="13">
         <v>46257</v>
@@ -4983,7 +5543,7 @@
         <v>46260</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="57">
@@ -4997,13 +5557,13 @@
         <v>32</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G5" s="13">
         <v>46257</v>
@@ -5019,12 +5579,12 @@
         <v>46260</v>
       </c>
       <c r="L5" s="17" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="42.75">
       <c r="A6" s="12" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B6">
         <v>220042034</v>
@@ -5033,13 +5593,13 @@
         <v>32</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G6" s="13">
         <v>46253</v>
@@ -5055,7 +5615,7 @@
         <v>46253</v>
       </c>
       <c r="L6" s="17" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="42.75">
@@ -5069,13 +5629,13 @@
         <v>32</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G7" s="13">
         <v>46254</v>
@@ -5091,7 +5651,7 @@
         <v>46264</v>
       </c>
       <c r="L7" s="17" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="42.75">
@@ -5105,32 +5665,30 @@
         <v>32</v>
       </c>
       <c r="D8" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="F8" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>183</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>182</v>
       </c>
       <c r="G8" s="13"/>
       <c r="H8" s="23">
         <v>0</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="J8" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="K8" s="13">
-        <v>46259</v>
-      </c>
+      <c r="K8" s="13"/>
       <c r="L8" s="17" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="57">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="28.5">
       <c r="A9" s="12" t="s">
         <v>151</v>
       </c>
@@ -5138,16 +5696,16 @@
         <v>222018199</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>325</v>
+        <v>289</v>
       </c>
       <c r="G9" s="13">
         <v>46289</v>
@@ -5157,9 +5715,7 @@
       <c r="J9" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="K9" s="13">
-        <v>46259</v>
-      </c>
+      <c r="K9" s="13"/>
       <c r="L9" s="17"/>
     </row>
     <row r="10" spans="1:12" ht="85.5">
@@ -5170,16 +5726,16 @@
         <v>221000537</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>326</v>
+        <v>290</v>
       </c>
       <c r="G10" s="13">
         <v>46274</v>
@@ -5189,29 +5745,27 @@
       <c r="J10" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="K10" s="13">
-        <v>46259</v>
-      </c>
+      <c r="K10" s="13"/>
       <c r="L10" s="17"/>
     </row>
     <row r="11" spans="1:12" ht="42.75">
       <c r="A11" s="12" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B11">
         <v>220042034</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G11" s="13">
         <v>46279</v>
@@ -5221,9 +5775,7 @@
       <c r="J11" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="K11" s="13">
-        <v>46259</v>
-      </c>
+      <c r="K11" s="13"/>
       <c r="L11" s="17"/>
     </row>
     <row r="12" spans="1:12" ht="42.75">
@@ -5234,13 +5786,13 @@
         <v>220049867</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>293</v>
@@ -5253,9 +5805,7 @@
       <c r="J12" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="K12" s="13">
-        <v>46259</v>
-      </c>
+      <c r="K12" s="13"/>
       <c r="L12" s="17"/>
     </row>
     <row r="13" spans="1:12" ht="28.5">
@@ -5266,10 +5816,10 @@
         <v>224131387</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E13" s="12" t="s">
         <v>294</v>
@@ -5285,9 +5835,7 @@
       <c r="J13" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="K13" s="13">
-        <v>46259</v>
-      </c>
+      <c r="K13" s="13"/>
       <c r="L13" s="17"/>
     </row>
     <row r="14" spans="1:12" ht="42.75">
@@ -5298,16 +5846,16 @@
         <v>224074632</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="G14" s="13">
         <v>46279</v>
@@ -5317,93 +5865,199 @@
       <c r="J14" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="K14" s="13">
-        <v>46259</v>
-      </c>
+      <c r="K14" s="13"/>
       <c r="L14" s="17"/>
     </row>
-    <row r="15" spans="1:12">
-      <c r="A15" s="16"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="13"/>
+    <row r="15" spans="1:12" ht="128.25">
+      <c r="A15" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="B15" s="12">
+        <v>222018199</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>422</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>423</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>424</v>
+      </c>
+      <c r="G15" s="13">
+        <v>46320</v>
+      </c>
       <c r="H15" s="23"/>
       <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="13"/>
+      <c r="J15" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="K15" s="13">
+        <v>46314</v>
+      </c>
       <c r="L15" s="17"/>
     </row>
-    <row r="16" spans="1:12">
-      <c r="A16" s="16"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="13"/>
+    <row r="16" spans="1:12" ht="128.25">
+      <c r="A16" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="B16" s="12">
+        <v>221000537</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>425</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>426</v>
+      </c>
+      <c r="G16" s="13">
+        <v>46318</v>
+      </c>
       <c r="H16" s="23"/>
       <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="13"/>
+      <c r="J16" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="K16" s="13">
+        <v>46311</v>
+      </c>
       <c r="L16" s="17"/>
     </row>
-    <row r="17" spans="1:12">
-      <c r="A17" s="16"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="13"/>
+    <row r="17" spans="1:12" ht="85.5">
+      <c r="A17" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="B17" s="12">
+        <v>224131387</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>427</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>428</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>429</v>
+      </c>
+      <c r="G17" s="13">
+        <v>46318</v>
+      </c>
       <c r="H17" s="23"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="13"/>
+      <c r="J17" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="K17" s="13">
+        <v>46312</v>
+      </c>
       <c r="L17" s="17"/>
     </row>
-    <row r="18" spans="1:12">
-      <c r="A18" s="16"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="13"/>
+    <row r="18" spans="1:12" ht="99.75">
+      <c r="A18" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="B18" s="12">
+        <v>220042034</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>432</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>433</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>434</v>
+      </c>
+      <c r="G18" s="13">
+        <v>46320</v>
+      </c>
       <c r="H18" s="23"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="13"/>
+      <c r="J18" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="K18" s="13">
+        <v>46312</v>
+      </c>
       <c r="L18" s="17"/>
     </row>
-    <row r="19" spans="1:12">
-      <c r="A19" s="16"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="13"/>
+    <row r="19" spans="1:12" ht="71.25">
+      <c r="A19" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="B19" s="12">
+        <v>220049867</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>336</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>430</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>431</v>
+      </c>
+      <c r="G19" s="13">
+        <v>46318</v>
+      </c>
       <c r="H19" s="23"/>
       <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="13"/>
+      <c r="J19" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="K19" s="13">
+        <v>46310</v>
+      </c>
       <c r="L19" s="17"/>
     </row>
-    <row r="20" spans="1:12">
-      <c r="A20" s="16"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="13"/>
+    <row r="20" spans="1:12" ht="71.25">
+      <c r="A20" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="B20" s="12">
+        <v>224074632</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>436</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>435</v>
+      </c>
+      <c r="G20" s="13">
+        <v>46318</v>
+      </c>
       <c r="H20" s="23"/>
       <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="13"/>
+      <c r="J20" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="K20" s="13">
+        <v>46312</v>
+      </c>
       <c r="L20" s="17"/>
     </row>
     <row r="21" spans="1:12">
@@ -7953,11 +8607,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="C3:C201" xr:uid="{00000000-0002-0000-0300-000000000000}">
-      <formula1>"Unit 1 / Phase 1,Phase 2,Phase 3,Final"</formula1>
-    </dataValidation>
     <dataValidation type="list" sqref="J3:J201" xr:uid="{00000000-0002-0000-0300-000001000000}">
       <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="C3:C201 D20" xr:uid="{00000000-0002-0000-0300-000000000000}">
+      <formula1>"Unit 1 / Phase 1,Phase 2,Phase 3,Final"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8034,7 +8688,7 @@
         <v>157</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E3" s="12" t="s">
         <v>158</v>
@@ -8046,10 +8700,10 @@
         <v>160</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="42.75">
@@ -8063,22 +8717,22 @@
         <v>157</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>161</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="85.5">
@@ -8086,25 +8740,25 @@
         <v>46279</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C5" s="12" t="s">
+        <v>301</v>
+      </c>
+      <c r="D5" s="12" t="s">
         <v>302</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="E5" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="G5" s="12" t="s">
         <v>303</v>
       </c>
-      <c r="E5" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>231</v>
-      </c>
-      <c r="G5" s="12" t="s">
+      <c r="H5" s="12" t="s">
         <v>304</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>305</v>
       </c>
       <c r="I5" s="17"/>
     </row>
@@ -8113,38 +8767,56 @@
         <v>46286</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D6" s="12" t="s">
+        <v>305</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="G6" s="12" t="s">
         <v>306</v>
       </c>
-      <c r="E6" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>231</v>
-      </c>
-      <c r="G6" s="12" t="s">
+      <c r="H6" s="12" t="s">
         <v>307</v>
       </c>
-      <c r="H6" s="12" t="s">
-        <v>308</v>
-      </c>
       <c r="I6" s="17"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="25"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="17"/>
+      <c r="A7" s="25">
+        <v>46318</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="C7" t="s">
+        <v>338</v>
+      </c>
+      <c r="D7" t="s">
+        <v>339</v>
+      </c>
+      <c r="E7" s="38" t="s">
+        <v>187</v>
+      </c>
+      <c r="F7" s="39" t="s">
+        <v>340</v>
+      </c>
+      <c r="G7" t="s">
+        <v>341</v>
+      </c>
+      <c r="H7" t="s">
+        <v>342</v>
+      </c>
+      <c r="I7" t="s">
+        <v>343</v>
+      </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="25"/>
@@ -9188,7 +9860,7 @@
     <dataValidation type="list" sqref="B3:B101" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Unit 1 / Phase 1,Phase 2,Phase 3,Final"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C3:C101" xr:uid="{00000000-0002-0000-0400-000001000000}">
+    <dataValidation type="list" sqref="C3:C6 C8:C101" xr:uid="{00000000-0002-0000-0400-000001000000}">
       <formula1>"Meeting,Telephone Call,Online Meeting,Email,Site Visit,Other"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9258,13 +9930,13 @@
         <v>32</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F3" s="12" t="s">
         <v>162</v>
@@ -9284,16 +9956,16 @@
         <v>32</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="G4" s="13">
         <v>46265</v>
@@ -9310,16 +9982,16 @@
         <v>32</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="G5" s="13">
         <v>46269</v>
@@ -9328,61 +10000,107 @@
         <v>163</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="42.75">
+    <row r="6" spans="1:8" ht="28.5">
       <c r="A6" s="25">
         <v>46276</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>322</v>
+        <v>296</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>323</v>
+        <v>297</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>324</v>
+        <v>298</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>296</v>
-      </c>
-      <c r="G6" s="13">
-        <v>46287</v>
-      </c>
+        <v>299</v>
+      </c>
+      <c r="G6" s="13"/>
       <c r="H6" s="17" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="25"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="17"/>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="25"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="17"/>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="25"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="17"/>
+    <row r="7" spans="1:8" ht="42.75">
+      <c r="A7" s="25">
+        <v>46299</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>319</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>320</v>
+      </c>
+      <c r="G7" s="13">
+        <v>46301</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="42.75">
+      <c r="A8" s="25">
+        <v>46311</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>321</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>323</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>324</v>
+      </c>
+      <c r="G8" s="13">
+        <v>46313</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="42.75">
+      <c r="A9" s="25">
+        <v>46316</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>344</v>
+      </c>
+      <c r="C9" t="s">
+        <v>345</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>346</v>
+      </c>
+      <c r="E9" t="s">
+        <v>347</v>
+      </c>
+      <c r="F9" t="s">
+        <v>249</v>
+      </c>
+      <c r="G9" s="13">
+        <v>46316</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="25"/>
@@ -10375,7 +11093,7 @@
         <v>53</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>32</v>
+        <v>308</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>108</v>
@@ -10389,7 +11107,7 @@
         <v>55</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>297</v>
+        <v>325</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>109</v>
@@ -10417,7 +11135,7 @@
         <v>112</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>298</v>
+        <v>326</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>113</v>
@@ -10431,7 +11149,7 @@
         <v>114</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>115</v>
@@ -10457,7 +11175,7 @@
         <v>118</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>299</v>
+        <v>327</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>119</v>
@@ -10471,7 +11189,7 @@
         <v>120</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>319</v>
+        <v>250</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>121</v>
@@ -10485,7 +11203,7 @@
         <v>122</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>249</v>
+        <v>164</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>123</v>
@@ -10499,7 +11217,7 @@
         <v>124</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>300</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -10571,7 +11289,7 @@
         <v>53</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>127</v>
@@ -10585,7 +11303,7 @@
         <v>47</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>129</v>
@@ -10599,7 +11317,7 @@
         <v>131</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>132</v>
@@ -10613,7 +11331,7 @@
         <v>134</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>135</v>
@@ -10627,7 +11345,7 @@
         <v>137</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>310</v>
+        <v>330</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>138</v>
@@ -10641,7 +11359,7 @@
         <v>140</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>312</v>
+        <v>331</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="74.099999999999994" customHeight="1">
@@ -10649,7 +11367,7 @@
         <v>141</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>313</v>
+        <v>332</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="74.099999999999994" customHeight="1">
@@ -10657,7 +11375,7 @@
         <v>142</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>314</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="74.099999999999994" customHeight="1">
@@ -10665,7 +11383,7 @@
         <v>143</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="74.099999999999994" customHeight="1">
@@ -10673,7 +11391,7 @@
         <v>144</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>316</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="74.099999999999994" customHeight="1">
@@ -10681,7 +11399,7 @@
         <v>145</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>317</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="74.099999999999994" customHeight="1">
@@ -10689,7 +11407,7 @@
         <v>146</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>318</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>